<commit_message>
Descarga de OTs entre el 05/01 y el 06/01
</commit_message>
<xml_diff>
--- a/Tipos de trabajo/output/resumen_trabajos.xlsx
+++ b/Tipos de trabajo/output/resumen_trabajos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dacm/we/odoo_con_trabajos/Tipos de trabajo/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57060C91-9467-934D-9D2F-72B7265D839F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4885F51A-AECB-BD41-B80E-C050331128FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-5560" windowWidth="33720" windowHeight="19920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37540" yWindow="-5520" windowWidth="33720" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="trabajos" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="226" r:id="rId3"/>
+    <pivotCache cacheId="258" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3825" uniqueCount="1162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3865" uniqueCount="1178">
   <si>
     <t>Técnico</t>
   </si>
@@ -4399,6 +4399,56 @@
 - Se hace entrega de documentación a Sr. Nicolas solicitado por Rodrigo López.
 - Se espero a don Diego Ramos para la verificación de instalación de los postes en los puntos PEM, pero no fue posible reunirnos, esta coordinado para hoy a las 10:00hrs apox.
 - Se rotula las herramientas acorde al color reactivo de este mes. </t>
+  </si>
+  <si>
+    <t>Configuración telemetria pozo BN12</t>
+  </si>
+  <si>
+    <t>Se intstala sensor de nivel en pozo y se configura el equipo junto con el flujometro a traves de lecturas modbus, se comprueban valores en PLC.
+Por otro lado se configura la comunicación del punto a la telemetria WeTechs para la visualizacion de datos.
+Adicionalmente se instalan equipos de comunicación para la lectura de datos a través de red LORA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migración a Red Lora Wan LT </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matias Signorio - Paula Riquelme </t>
+  </si>
+  <si>
+    <t>Se instalan y configuración dispositivo red Lora Wan, se validan datos terreno plataforma ok + antena ok.</t>
+  </si>
+  <si>
+    <t>Uc300-915M</t>
+  </si>
+  <si>
+    <t>6445F17824030004</t>
+  </si>
+  <si>
+    <t>Punto ok.</t>
+  </si>
+  <si>
+    <t>[Global Tórtolas] Pozo BN1</t>
+  </si>
+  <si>
+    <t>Se instalan y configuración dispositivo red Lora Wan, se validan datos terreno plataforma ok. + antena</t>
+  </si>
+  <si>
+    <t>6445F15707350005</t>
+  </si>
+  <si>
+    <t>Punto transmisión de datos ok.</t>
+  </si>
+  <si>
+    <t>Se instalan y configuración dispositivo red Lora Wan, se validan datos terreno plataforma ok. + antena ok.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uc300-915M </t>
+  </si>
+  <si>
+    <t>6445F15534110005</t>
+  </si>
+  <si>
+    <t>Punto con transmisión de datos ok.</t>
   </si>
 </sst>
 </file>
@@ -4459,7 +4509,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4472,7 +4522,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13618,7 +13667,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{58C144FF-F8BA-0042-8CC8-638EF8B29700}" name="Resumen" cacheId="226" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{58C144FF-F8BA-0042-8CC8-638EF8B29700}" name="Resumen" cacheId="258" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="A1:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField dataField="1" showAll="0"/>
@@ -13790,14 +13839,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{32CCDECC-D932-5D4F-9FF6-DAB914B6B73F}" name="Tabla1" displayName="Tabla1" ref="A1:N466" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="A1:N466" xr:uid="{32CCDECC-D932-5D4F-9FF6-DAB914B6B73F}">
-    <filterColumn colId="6">
-      <filters>
-        <dateGroupItem year="2025" dateTimeGrouping="year"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{32CCDECC-D932-5D4F-9FF6-DAB914B6B73F}" name="Tabla1" displayName="Tabla1" ref="A1:N470" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A1:N470" xr:uid="{32CCDECC-D932-5D4F-9FF6-DAB914B6B73F}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A33:N422">
     <sortCondition descending="1" ref="E1:E466"/>
   </sortState>
@@ -14106,7 +14149,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N466"/>
+  <dimension ref="A1:N470"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
@@ -30580,7 +30623,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="464" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="464" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A464">
         <v>366</v>
       </c>
@@ -30621,7 +30664,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="465" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="465" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A465">
         <v>368</v>
       </c>
@@ -30653,7 +30696,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="466" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="466" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A466">
         <v>368</v>
       </c>
@@ -30683,6 +30726,170 @@
       </c>
       <c r="J466">
         <v>5</v>
+      </c>
+    </row>
+    <row r="467" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A467">
+        <v>369</v>
+      </c>
+      <c r="B467" t="s">
+        <v>67</v>
+      </c>
+      <c r="C467" t="s">
+        <v>1162</v>
+      </c>
+      <c r="D467" t="s">
+        <v>63</v>
+      </c>
+      <c r="E467" t="s">
+        <v>1128</v>
+      </c>
+      <c r="F467" t="s">
+        <v>17</v>
+      </c>
+      <c r="G467" s="1">
+        <v>46028</v>
+      </c>
+      <c r="H467" t="s">
+        <v>479</v>
+      </c>
+      <c r="I467" t="s">
+        <v>1163</v>
+      </c>
+      <c r="J467">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="468" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A468">
+        <v>370</v>
+      </c>
+      <c r="B468" t="s">
+        <v>113</v>
+      </c>
+      <c r="C468" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D468" t="s">
+        <v>63</v>
+      </c>
+      <c r="E468" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F468" t="s">
+        <v>227</v>
+      </c>
+      <c r="G468" s="1">
+        <v>46028</v>
+      </c>
+      <c r="H468" t="s">
+        <v>1165</v>
+      </c>
+      <c r="I468" t="s">
+        <v>1166</v>
+      </c>
+      <c r="J468">
+        <v>5</v>
+      </c>
+      <c r="K468" t="s">
+        <v>209</v>
+      </c>
+      <c r="L468" t="s">
+        <v>1167</v>
+      </c>
+      <c r="M468" t="s">
+        <v>1168</v>
+      </c>
+      <c r="N468" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="469" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A469">
+        <v>370</v>
+      </c>
+      <c r="B469" t="s">
+        <v>113</v>
+      </c>
+      <c r="C469" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D469" t="s">
+        <v>63</v>
+      </c>
+      <c r="E469" t="s">
+        <v>1170</v>
+      </c>
+      <c r="F469" t="s">
+        <v>227</v>
+      </c>
+      <c r="G469" s="1">
+        <v>46028</v>
+      </c>
+      <c r="H469" t="s">
+        <v>1165</v>
+      </c>
+      <c r="I469" t="s">
+        <v>1171</v>
+      </c>
+      <c r="J469">
+        <v>5</v>
+      </c>
+      <c r="K469" t="s">
+        <v>209</v>
+      </c>
+      <c r="L469" t="s">
+        <v>1167</v>
+      </c>
+      <c r="M469" t="s">
+        <v>1172</v>
+      </c>
+      <c r="N469" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="470" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A470">
+        <v>370</v>
+      </c>
+      <c r="B470" t="s">
+        <v>113</v>
+      </c>
+      <c r="C470" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D470" t="s">
+        <v>63</v>
+      </c>
+      <c r="E470" t="s">
+        <v>1128</v>
+      </c>
+      <c r="F470" t="s">
+        <v>227</v>
+      </c>
+      <c r="G470" s="1">
+        <v>46028</v>
+      </c>
+      <c r="H470" t="s">
+        <v>1165</v>
+      </c>
+      <c r="I470" t="s">
+        <v>1174</v>
+      </c>
+      <c r="J470">
+        <v>5</v>
+      </c>
+      <c r="K470" t="s">
+        <v>209</v>
+      </c>
+      <c r="L470" t="s">
+        <v>1175</v>
+      </c>
+      <c r="M470" t="s">
+        <v>1176</v>
+      </c>
+      <c r="N470" t="s">
+        <v>1177</v>
       </c>
     </row>
   </sheetData>
@@ -30715,7 +30922,7 @@
       <c r="A2" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2">
         <v>14</v>
       </c>
     </row>
@@ -30723,7 +30930,7 @@
       <c r="A3" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3">
         <v>4</v>
       </c>
     </row>
@@ -30731,7 +30938,7 @@
       <c r="A4" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4">
         <v>94</v>
       </c>
     </row>
@@ -30739,7 +30946,7 @@
       <c r="A5" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5">
         <v>50</v>
       </c>
     </row>
@@ -30747,7 +30954,7 @@
       <c r="A6" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6">
         <v>20</v>
       </c>
     </row>
@@ -30755,7 +30962,7 @@
       <c r="A7" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7">
         <v>33</v>
       </c>
     </row>
@@ -30763,7 +30970,7 @@
       <c r="A8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8">
         <v>247</v>
       </c>
     </row>
@@ -30771,7 +30978,7 @@
       <c r="A9" s="5" t="s">
         <v>1138</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9">
         <v>462</v>
       </c>
     </row>

</xml_diff>